<commit_message>
🐛 Fix Prisma connection pool limit on Vercel
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_pacientes.xlsx
+++ b/public/templates/plantilla_pacientes.xlsx
@@ -1,41 +1,176 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeanp\Documents\registro\public\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332EBD92-4414-428D-8052-18C16BCBE1F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Usuarios" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="48">
+  <si>
+    <t>Nombre Completo</t>
+  </si>
+  <si>
+    <t>DNI</t>
+  </si>
+  <si>
+    <t>Rol</t>
+  </si>
+  <si>
+    <t>Sede (Opcional)</t>
+  </si>
+  <si>
+    <t>PACIENTE_SIMULADO</t>
+  </si>
+  <si>
+    <t>Campus Villa</t>
+  </si>
+  <si>
+    <t>Andrea Victoria García Carrasco</t>
+  </si>
+  <si>
+    <t>Anthony Mauro Ramos Espinoza</t>
+  </si>
+  <si>
+    <t>Brissa Molina</t>
+  </si>
+  <si>
+    <t>Edwin David Puma Castillo</t>
+  </si>
+  <si>
+    <t>Luis Fernando Capitan Campa</t>
+  </si>
+  <si>
+    <t>Sally Nicole Kling Marín</t>
+  </si>
+  <si>
+    <t>Juliet Rashell Pacahuala Mallqui</t>
+  </si>
+  <si>
+    <t>Leonora Maurial Mackee</t>
+  </si>
+  <si>
+    <t>Piero Espinoza Flores</t>
+  </si>
+  <si>
+    <t>Rubí Yessenia Cáceres Puma</t>
+  </si>
+  <si>
+    <t>Sara Elizabeth Puma castillo</t>
+  </si>
+  <si>
+    <t>Sergio Marroquin</t>
+  </si>
+  <si>
+    <t>Anabell Quispe Huayta</t>
+  </si>
+  <si>
+    <t>José Alejandro Parreño Angulo</t>
+  </si>
+  <si>
+    <t>Josefa Arellano Grandez</t>
+  </si>
+  <si>
+    <t>Joselyn Pozo Quispe</t>
+  </si>
+  <si>
+    <t>Lisbett Yulian Puma Gutiérrez</t>
+  </si>
+  <si>
+    <t>Mery Lucía Ludena perez</t>
+  </si>
+  <si>
+    <t>Rosa Puma Castillo</t>
+  </si>
+  <si>
+    <t>Silvia Franco Fernandez de Fernandez</t>
+  </si>
+  <si>
+    <t>Wendy Liz Gutierrrez Coba</t>
+  </si>
+  <si>
+    <t>Zayda Consuelo Cayo ortiz</t>
+  </si>
+  <si>
+    <t>Beatriz Guerra Cóndor</t>
+  </si>
+  <si>
+    <t>Carmen Rosa Ludeña Palomino</t>
+  </si>
+  <si>
+    <t>Haydee Eva Deza Chavarria</t>
+  </si>
+  <si>
+    <t>Dina Felicita Cáceres Enciso</t>
+  </si>
+  <si>
+    <t>Henry André Mansilla Sánchez</t>
+  </si>
+  <si>
+    <t>Javier Tapia Silva</t>
+  </si>
+  <si>
+    <t>Neldo Ernesto Tapia Silva</t>
+  </si>
+  <si>
+    <t>Marisa Calla Sarmiento</t>
+  </si>
+  <si>
+    <t>Leo Gerardo Gómez Fernua</t>
+  </si>
+  <si>
+    <t>Miriam Gracy Robles Puma</t>
+  </si>
+  <si>
+    <t>Milagros Obeso Aguirre</t>
+  </si>
+  <si>
+    <t>Angelo Cáceres puma</t>
+  </si>
+  <si>
+    <t>Joe André Silva Lazo</t>
+  </si>
+  <si>
+    <t>MAURICIO ALBERTO ARMAS BEST</t>
+  </si>
+  <si>
+    <t>KLEDY BENJAMIN DONGO PFLUCKER</t>
+  </si>
+  <si>
+    <t>06267231</t>
+  </si>
+  <si>
+    <t>09130167</t>
+  </si>
+  <si>
+    <t>09625066</t>
+  </si>
+  <si>
+    <t>07899948</t>
+  </si>
+  <si>
+    <t>07856095</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -43,16 +178,52 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF1E293B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF242424"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,18 +231,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,54 +610,548 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D39"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.09765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.09765625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Nombre Completo</v>
-      </c>
-      <c r="B1" t="str">
-        <v>DNI</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Rol</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Sede (Opcional)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Ejemplo Nombre 1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>11111111</v>
-      </c>
-      <c r="C2" t="str">
-        <v>PACIENTE_SIMULADO</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Campus Villa</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Ejemplo Nombre 2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>22222222</v>
-      </c>
-      <c r="C3" t="str">
-        <v>PACIENTE_SIMULADO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Campus Norte</v>
-      </c>
-    </row>
+    <row r="1" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="4">
+        <v>45195178</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4">
+        <v>43504880</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="5">
+        <v>76877590</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="4">
+        <v>40090505</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="5">
+        <v>74068325</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="4">
+        <v>70265383</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="5">
+        <v>75228772</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="4">
+        <v>10553728</v>
+      </c>
+      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="4">
+        <v>75495902</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="4">
+        <v>44293279</v>
+      </c>
+      <c r="C11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="4">
+        <v>10648160</v>
+      </c>
+      <c r="C12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="5">
+        <v>45923220</v>
+      </c>
+      <c r="C13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="4">
+        <v>40880104</v>
+      </c>
+      <c r="C14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="4">
+        <v>41561761</v>
+      </c>
+      <c r="C15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="4">
+        <v>44979340</v>
+      </c>
+      <c r="C16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="5">
+        <v>48298225</v>
+      </c>
+      <c r="C17" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="5">
+        <v>42711339</v>
+      </c>
+      <c r="C18" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="4">
+        <v>45784931</v>
+      </c>
+      <c r="C19" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
+        <v>4</v>
+      </c>
+      <c r="D20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="5">
+        <v>47709220</v>
+      </c>
+      <c r="C22" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="4">
+        <v>45797213</v>
+      </c>
+      <c r="C23" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="4">
+        <v>44160018</v>
+      </c>
+      <c r="C25" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="5">
+        <v>19238316</v>
+      </c>
+      <c r="C26" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="5">
+        <v>40358302</v>
+      </c>
+      <c r="C27" t="s">
+        <v>4</v>
+      </c>
+      <c r="D27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="4">
+        <v>10015187</v>
+      </c>
+      <c r="C28" t="s">
+        <v>4</v>
+      </c>
+      <c r="D28" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" t="s">
+        <v>4</v>
+      </c>
+      <c r="D29" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" t="s">
+        <v>4</v>
+      </c>
+      <c r="D30" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" s="4">
+        <v>40000645</v>
+      </c>
+      <c r="C31" t="s">
+        <v>4</v>
+      </c>
+      <c r="D31" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="5">
+        <v>75329865</v>
+      </c>
+      <c r="C32" t="s">
+        <v>4</v>
+      </c>
+      <c r="D32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" s="4">
+        <v>40184523</v>
+      </c>
+      <c r="C33" t="s">
+        <v>4</v>
+      </c>
+      <c r="D33" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34" s="5">
+        <v>70528938</v>
+      </c>
+      <c r="C34" t="s">
+        <v>4</v>
+      </c>
+      <c r="D34" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="4">
+        <v>76827272</v>
+      </c>
+      <c r="C35" t="s">
+        <v>4</v>
+      </c>
+      <c r="D35" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36" s="6"/>
+      <c r="C36" t="s">
+        <v>4</v>
+      </c>
+      <c r="D36" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B37" s="5">
+        <v>80373084</v>
+      </c>
+      <c r="C37" t="s">
+        <v>4</v>
+      </c>
+      <c r="D37" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C38" t="s">
+        <v>4</v>
+      </c>
+      <c r="D38" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15.6" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError sqref="A1:D1 C2:D2 C3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>